<commit_message>
feat: adiciona diretrizes de acessibilidade e neurodivergência (TEA)
Nova aba Acessibilidade_e_Confissao na planilha regrasdeouro.xlsx:
- Linguagem literal obrigatória (sem metáforas idiomáticas)
- Comandos objetivos e estruturados (sem subjetividade)
- Proibição de rótulos negativos para crianças
- Identidade religiosa: apenas referências cristãs evangélicas
- Versão bíblica padronizada: NVI exclusivamente
- Instruções segmentadas para reduzir carga sensorial (TEA)
- Proibição de ironia/sarcasmo em diálogos

CLAUDE.md atualizado com seção 6 completa.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/regrasdeouro.xlsx
+++ b/dados/regrasdeouro.xlsx
@@ -7,6 +7,7 @@
     <sheet state="visible" name="Proibicao_e_Restricao" sheetId="2" r:id="rId6"/>
     <sheet state="visible" name="Diretrizes_Editor_IA" sheetId="3" r:id="rId7"/>
     <sheet state="visible" name="Diretrizes_Manual_Professor" sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="Acessibilidade_e_Confissao" sheetId="5" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -14,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="322">
   <si>
     <t>Ano Escolar</t>
   </si>
@@ -890,6 +891,96 @@
   </si>
   <si>
     <t>Citar a obra e o porquê da indicação para o tema.</t>
+  </si>
+  <si>
+    <t>O que EVITAR (Risco)</t>
+  </si>
+  <si>
+    <t>O que USAR (Padrão Ouro)</t>
+  </si>
+  <si>
+    <t>Justificativa (TEA / Confessional)</t>
+  </si>
+  <si>
+    <t>Linguagem Literal (TEA)</t>
+  </si>
+  <si>
+    <t>Metáforas e expressões idiomáticas (Ex: 'Bate mais forte', 'Choveu canivete', 'Caiu a ficha').</t>
+  </si>
+  <si>
+    <t>Linguagem direta e acadêmica (Ex: 'Aplique mais força', 'Choveu muito', 'Entendeu o conceito').</t>
+  </si>
+  <si>
+    <t>Crianças com TEA podem interpretar metáforas literalmente, gerando confusão, medo ou comportamentos inadequados (ex: agressividade física).</t>
+  </si>
+  <si>
+    <t>Comandos subjetivos (Ex: 'Use sua imaginação', 'Faça como quiser').</t>
+  </si>
+  <si>
+    <t>Comandos objetivos e estruturados (Ex: 'Desenhe um animal que você conhece', 'Siga o passo a passo').</t>
+  </si>
+  <si>
+    <t>A subjetividade excessiva pode causar ansiedade e travamento cognitivo em crianças atípicas.</t>
+  </si>
+  <si>
+    <t>Rótulos e Estigmas</t>
+  </si>
+  <si>
+    <t>Adjetivos pejorativos ou espiritualmente carregados (Ex: 'Criança endiabrada', 'Menino difícil').</t>
+  </si>
+  <si>
+    <t>Descrição de comportamento ou potencial (Ex: 'Criança com muita energia', 'Estudante em desenvolvimento').</t>
+  </si>
+  <si>
+    <t>Termos como 'endiabrado' são ofensivos e ferem a cosmovisão cristã, além de rotular negativamente a criança.</t>
+  </si>
+  <si>
+    <t>Identidade Religiosa</t>
+  </si>
+  <si>
+    <t>Santos católicos, personagens da hagiografia ou estímulos sincréticos (Ex: Fitinhas do Bonfim, imagens de santos).</t>
+  </si>
+  <si>
+    <t>Personagens bíblicos, heróis da fé cristã evangélica ou elementos neutros da natureza.</t>
+  </si>
+  <si>
+    <t>O material é para uma rede cristã evangélica. Elementos de outras vertentes religiosas causam estranheza e não pertencimento.</t>
+  </si>
+  <si>
+    <t>Padronização Bíblica</t>
+  </si>
+  <si>
+    <t>Citações de versões variadas (Almeida, Ave Maria, NTLH).</t>
+  </si>
+  <si>
+    <t>Uso exclusivo da Versão NVI (Nova Versão Internacional).</t>
+  </si>
+  <si>
+    <t>Garante unidade doutrinária e linguagem contemporânea acessível à criança e à família.</t>
+  </si>
+  <si>
+    <t>Carga Sensorial (TEA)</t>
+  </si>
+  <si>
+    <t>Instruções com excesso de estímulos visuais ou auditivos descritos de forma caótica.</t>
+  </si>
+  <si>
+    <t>Instruções segmentadas, com apoio visual claro e listas numeradas.</t>
+  </si>
+  <si>
+    <t>Reduz a sobrecarga sensorial e facilita a organização mental do estudante atípico.</t>
+  </si>
+  <si>
+    <t>Interação Social</t>
+  </si>
+  <si>
+    <t>Ironia ou sarcasmo em diálogos de personagens.</t>
+  </si>
+  <si>
+    <t>Diálogos honestos, claros e exemplares.</t>
+  </si>
+  <si>
+    <t>A ironia é de difícil compreensão para crianças no espectro e pode ensinar modelos de comunicação ineficientes.</t>
   </si>
 </sst>
 </file>
@@ -915,7 +1006,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -952,6 +1043,12 @@
         <bgColor rgb="FF38761D"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3D85C6"/>
+        <bgColor rgb="FF3D85C6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -959,7 +1056,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -987,6 +1084,9 @@
     <xf borderId="0" fillId="6" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1008,6 +1108,10 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -2309,4 +2413,133 @@
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="18.88"/>
+    <col customWidth="1" min="2" max="3" width="31.38"/>
+    <col customWidth="1" min="4" max="4" width="37.63"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>292</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>321</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: adiciona diretrizes de Humanidades Cristãs (cosmovisão x BNCC)
Nova seção 6 no CLAUDE.md — aba Humanidades_Cristas da planilha:
- Conteúdos BNCC obrigatórios devem ser incluídos mas contextualizados
- Teorias naturalistas apresentadas como "modelos" ou "visões", não verdades absolutas
- Contraponto da cosmovisão cristã obrigatório em: evolução, Big Bang,
  iluminismo, sociologia da religião, relativismo moral e arte
- Expressões-chave padronizadas: "Segundo esta teoria...", "A cosmovisão
  cristã compreende que...", "Sob esta perspectiva..."

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/regrasdeouro.xlsx
+++ b/dados/regrasdeouro.xlsx
@@ -4,10 +4,11 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Diretrizes_Anos_Escolares" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Proibicao_e_Restricao" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Diretrizes_Editor_IA" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="Diretrizes_Manual_Professor" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="Acessibilidade_e_Confissao" sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="Humanidades_Cristas" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="Proibicao_e_Restricao" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="Diretrizes_Editor_IA" sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="Diretrizes_Manual_Professor" sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="Acessibilidade_e_Confissao" sheetId="6" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -15,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="357">
   <si>
     <t>Ano Escolar</t>
   </si>
@@ -327,6 +328,111 @@
   </si>
   <si>
     <t>Máximo: Profundidade e interdisciplinaridade</t>
+  </si>
+  <si>
+    <t>Tema/Tópico</t>
+  </si>
+  <si>
+    <t>Conteúdo Obrigatório (BNCC)</t>
+  </si>
+  <si>
+    <t>Abordagem da Cosmovisão Cristã</t>
+  </si>
+  <si>
+    <t>Expressões Chave para o Texto</t>
+  </si>
+  <si>
+    <t>O que Evitar</t>
+  </si>
+  <si>
+    <t>Origem da Humanidade</t>
+  </si>
+  <si>
+    <t>Teoria da Evolução e ancestrais comuns.</t>
+  </si>
+  <si>
+    <t>Apresentar como um modelo científico de interpretação biológica, contrapondo com a doutrina da Criação divina.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 'Segundo a teoria evolutiva...', 'Sob a ótica científica naturalista...', 'A cosmovisão cristã compreende que...'</t>
+  </si>
+  <si>
+    <t>Afirmar que o homem 'veio do macaco' como um fato absoluto e único.</t>
+  </si>
+  <si>
+    <t>Surgimento do Universo</t>
+  </si>
+  <si>
+    <t>Teoria do Big Bang.</t>
+  </si>
+  <si>
+    <t>Expor a teoria como uma tentativa de explicar a mecânica da criação, mantendo Deus como a Causa Primária.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 'Cientistas propõem que...', 'Este modelo busca explicar...', 'Cremos que a ordem do universo reflete a sabedoria do Criador.'</t>
+  </si>
+  <si>
+    <t>Tratar o Big Bang como um evento puramente aleatório e sem propósito.</t>
+  </si>
+  <si>
+    <t>Filosofia Iluminista</t>
+  </si>
+  <si>
+    <t>Antropocentrismo e a Razão como guia única.</t>
+  </si>
+  <si>
+    <t>Valorizar a razão como dom de Deus, mas apontar a falibilidade humana sem a direção divina.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 'Os filósofos iluministas defendiam...', 'Embora a razão seja essencial, a fé oferece o sentido último...'</t>
+  </si>
+  <si>
+    <t>Validar que 'o homem é a medida de todas as coisas' sem ressalvas teológicas.</t>
+  </si>
+  <si>
+    <t>Sociologia e Religião</t>
+  </si>
+  <si>
+    <t>Religião como construção social ou 'ópio'.</t>
+  </si>
+  <si>
+    <t>Apresentar as visões de Marx/Durkheim como análises sociológicas de sua época, reafirmando a fé como verdade espiritual.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 'Para este pensador, a religião era...', 'Diferente desta visão sociológica, a experiência cristã baseia-se em...'</t>
+  </si>
+  <si>
+    <t>Tratar a fé apenas como um fenômeno cultural ou ferramenta de controle social.</t>
+  </si>
+  <si>
+    <t>Ética e Moral</t>
+  </si>
+  <si>
+    <t>Relativismo moral e construções culturais.</t>
+  </si>
+  <si>
+    <t>Expor as diferentes culturas, mas fundamentar a ética nos valores absolutos e eternos da Bíblia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 'Embora sociedades tenham normas diferentes, os princípios bíblicos nos chamam a...', 'Valores como justiça e amor transcendem culturas...'</t>
+  </si>
+  <si>
+    <t>Afirmar que 'não existe certo ou errado absoluto'.</t>
+  </si>
+  <si>
+    <t>Arte e Expressão</t>
+  </si>
+  <si>
+    <t>Arte como ruptura e questionamento de valores.</t>
+  </si>
+  <si>
+    <t>Celebrar a arte como reflexo da beleza de Deus (Beleza, Bondade e Verdade).</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 'A arte manifesta o dom criativo dado por Deus...', 'Esta obra propõe uma crítica que podemos analisar à luz de...'</t>
+  </si>
+  <si>
+    <t>Promover obras que profanam símbolos cristãos sem uma análise crítica e contextualizada.</t>
   </si>
   <si>
     <t>Categoria</t>
@@ -1006,7 +1112,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1017,6 +1123,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF4A86E8"/>
         <bgColor rgb="FF4A86E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF783F04"/>
+        <bgColor rgb="FF783F04"/>
       </patternFill>
     </fill>
     <fill>
@@ -1056,7 +1168,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1075,16 +1187,19 @@
     <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="6" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="8" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -1112,6 +1227,10 @@
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -1701,8 +1820,10 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="18.88"/>
-    <col customWidth="1" min="2" max="3" width="31.38"/>
-    <col customWidth="1" min="4" max="4" width="37.63"/>
+    <col customWidth="1" min="2" max="2" width="31.38"/>
+    <col customWidth="1" min="3" max="3" width="37.63"/>
+    <col customWidth="1" min="4" max="4" width="31.38"/>
+    <col customWidth="1" min="5" max="5" width="25.13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1718,173 +1839,110 @@
       <c r="D1" s="3" t="s">
         <v>107</v>
       </c>
+      <c r="E1" s="3" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>115</v>
+        <v>117</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>118</v>
+        <v>122</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>122</v>
+        <v>127</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>126</v>
+        <v>132</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="C9" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>138</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -1893,6 +1951,205 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="18.88"/>
+    <col customWidth="1" min="2" max="3" width="31.38"/>
+    <col customWidth="1" min="4" max="4" width="37.63"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>189</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -1908,283 +2165,283 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>159</v>
+      <c r="A1" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>165</v>
+      <c r="A2" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>171</v>
+      <c r="A3" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="C4" s="6" t="s">
+      <c r="A4" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>200</v>
+      <c r="C8" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>206</v>
+      <c r="A9" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>212</v>
+      <c r="A10" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>217</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>218</v>
+      <c r="A11" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>223</v>
+      <c r="A12" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>226</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>228</v>
+      <c r="A13" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>232</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>233</v>
+      <c r="A14" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -2192,7 +2449,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2207,207 +2464,207 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="s">
-        <v>234</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>235</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>236</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>237</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>238</v>
+      <c r="A1" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>243</v>
+      <c r="A2" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>246</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>248</v>
+      <c r="A3" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>249</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>253</v>
+      <c r="A4" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>254</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>257</v>
+      <c r="A5" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>260</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>261</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>262</v>
+      <c r="A6" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>264</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>266</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>267</v>
+      <c r="A7" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>269</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>270</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>272</v>
+      <c r="A8" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>304</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="s">
-        <v>273</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>274</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>277</v>
+      <c r="A9" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>310</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="s">
-        <v>278</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>279</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>280</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>282</v>
+      <c r="A10" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>284</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>285</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>286</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>287</v>
+      <c r="A11" s="7" t="s">
+        <v>318</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="s">
-        <v>288</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>289</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>290</v>
-      </c>
-      <c r="D12" s="6" t="s">
+      <c r="A12" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="E12" s="6" t="s">
-        <v>291</v>
+      <c r="E12" s="7" t="s">
+        <v>326</v>
       </c>
     </row>
   </sheetData>
@@ -2415,7 +2672,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2428,115 +2685,115 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>292</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>294</v>
+      <c r="A1" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>327</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>328</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>295</v>
+        <v>330</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>296</v>
+        <v>331</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>297</v>
+        <v>332</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>298</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>295</v>
+        <v>330</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>299</v>
+        <v>334</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>300</v>
+        <v>335</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>301</v>
+        <v>336</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>302</v>
+        <v>337</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>303</v>
+        <v>338</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>304</v>
+        <v>339</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>305</v>
+        <v>340</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>306</v>
+        <v>341</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>307</v>
+        <v>342</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>308</v>
+        <v>343</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>309</v>
+        <v>344</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
-        <v>310</v>
+        <v>345</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>311</v>
+        <v>346</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>312</v>
+        <v>347</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>313</v>
+        <v>348</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
-        <v>314</v>
+        <v>349</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>315</v>
+        <v>350</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>316</v>
+        <v>351</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>317</v>
+        <v>352</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
-        <v>318</v>
+        <v>353</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>319</v>
+        <v>354</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>320</v>
+        <v>355</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sync: incorpora estado atual da EC2 ao git
</commit_message>
<xml_diff>
--- a/dados/regrasdeouro.xlsx
+++ b/dados/regrasdeouro.xlsx
@@ -4,11 +4,10 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Diretrizes_Anos_Escolares" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Humanidades_Cristas" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Proibicao_e_Restricao" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="Diretrizes_Editor_IA" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="Diretrizes_Manual_Professor" sheetId="5" r:id="rId9"/>
-    <sheet state="visible" name="Acessibilidade_e_Confissao" sheetId="6" r:id="rId10"/>
+    <sheet state="visible" name="Proibicao_e_Restricao" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="Diretrizes_Editor_IA" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="Diretrizes_Manual_Professor" sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="Acessibilidade_e_Confissao" sheetId="5" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -16,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="322">
   <si>
     <t>Ano Escolar</t>
   </si>
@@ -328,111 +327,6 @@
   </si>
   <si>
     <t>Máximo: Profundidade e interdisciplinaridade</t>
-  </si>
-  <si>
-    <t>Tema/Tópico</t>
-  </si>
-  <si>
-    <t>Conteúdo Obrigatório (BNCC)</t>
-  </si>
-  <si>
-    <t>Abordagem da Cosmovisão Cristã</t>
-  </si>
-  <si>
-    <t>Expressões Chave para o Texto</t>
-  </si>
-  <si>
-    <t>O que Evitar</t>
-  </si>
-  <si>
-    <t>Origem da Humanidade</t>
-  </si>
-  <si>
-    <t>Teoria da Evolução e ancestrais comuns.</t>
-  </si>
-  <si>
-    <t>Apresentar como um modelo científico de interpretação biológica, contrapondo com a doutrina da Criação divina.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 'Segundo a teoria evolutiva...', 'Sob a ótica científica naturalista...', 'A cosmovisão cristã compreende que...'</t>
-  </si>
-  <si>
-    <t>Afirmar que o homem 'veio do macaco' como um fato absoluto e único.</t>
-  </si>
-  <si>
-    <t>Surgimento do Universo</t>
-  </si>
-  <si>
-    <t>Teoria do Big Bang.</t>
-  </si>
-  <si>
-    <t>Expor a teoria como uma tentativa de explicar a mecânica da criação, mantendo Deus como a Causa Primária.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 'Cientistas propõem que...', 'Este modelo busca explicar...', 'Cremos que a ordem do universo reflete a sabedoria do Criador.'</t>
-  </si>
-  <si>
-    <t>Tratar o Big Bang como um evento puramente aleatório e sem propósito.</t>
-  </si>
-  <si>
-    <t>Filosofia Iluminista</t>
-  </si>
-  <si>
-    <t>Antropocentrismo e a Razão como guia única.</t>
-  </si>
-  <si>
-    <t>Valorizar a razão como dom de Deus, mas apontar a falibilidade humana sem a direção divina.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 'Os filósofos iluministas defendiam...', 'Embora a razão seja essencial, a fé oferece o sentido último...'</t>
-  </si>
-  <si>
-    <t>Validar que 'o homem é a medida de todas as coisas' sem ressalvas teológicas.</t>
-  </si>
-  <si>
-    <t>Sociologia e Religião</t>
-  </si>
-  <si>
-    <t>Religião como construção social ou 'ópio'.</t>
-  </si>
-  <si>
-    <t>Apresentar as visões de Marx/Durkheim como análises sociológicas de sua época, reafirmando a fé como verdade espiritual.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 'Para este pensador, a religião era...', 'Diferente desta visão sociológica, a experiência cristã baseia-se em...'</t>
-  </si>
-  <si>
-    <t>Tratar a fé apenas como um fenômeno cultural ou ferramenta de controle social.</t>
-  </si>
-  <si>
-    <t>Ética e Moral</t>
-  </si>
-  <si>
-    <t>Relativismo moral e construções culturais.</t>
-  </si>
-  <si>
-    <t>Expor as diferentes culturas, mas fundamentar a ética nos valores absolutos e eternos da Bíblia.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 'Embora sociedades tenham normas diferentes, os princípios bíblicos nos chamam a...', 'Valores como justiça e amor transcendem culturas...'</t>
-  </si>
-  <si>
-    <t>Afirmar que 'não existe certo ou errado absoluto'.</t>
-  </si>
-  <si>
-    <t>Arte e Expressão</t>
-  </si>
-  <si>
-    <t>Arte como ruptura e questionamento de valores.</t>
-  </si>
-  <si>
-    <t>Celebrar a arte como reflexo da beleza de Deus (Beleza, Bondade e Verdade).</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 'A arte manifesta o dom criativo dado por Deus...', 'Esta obra propõe uma crítica que podemos analisar à luz de...'</t>
-  </si>
-  <si>
-    <t>Promover obras que profanam símbolos cristãos sem uma análise crítica e contextualizada.</t>
   </si>
   <si>
     <t>Categoria</t>
@@ -1112,7 +1006,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1123,12 +1017,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF4A86E8"/>
         <bgColor rgb="FF4A86E8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF783F04"/>
-        <bgColor rgb="FF783F04"/>
       </patternFill>
     </fill>
     <fill>
@@ -1168,7 +1056,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1187,19 +1075,16 @@
     <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="6" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="8" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -1227,10 +1112,6 @@
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -1820,10 +1701,8 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="18.88"/>
-    <col customWidth="1" min="2" max="2" width="31.38"/>
-    <col customWidth="1" min="3" max="3" width="37.63"/>
-    <col customWidth="1" min="4" max="4" width="31.38"/>
-    <col customWidth="1" min="5" max="5" width="25.13"/>
+    <col customWidth="1" min="2" max="3" width="31.38"/>
+    <col customWidth="1" min="4" max="4" width="37.63"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1839,110 +1718,173 @@
       <c r="D1" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>108</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>111</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>115</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="B7" s="4" t="s">
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="B9" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>138</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -1951,205 +1893,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="18.88"/>
-    <col customWidth="1" min="2" max="3" width="31.38"/>
-    <col customWidth="1" min="4" max="4" width="37.63"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>189</v>
-      </c>
-    </row>
-  </sheetData>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2165,283 +1908,283 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B7" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="C1" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="C2" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D8" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E8" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F8" s="6" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="7" t="s">
+    <row r="9">
+      <c r="A9" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B9" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C9" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D9" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E9" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F9" s="6" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="7" t="s">
+    <row r="10">
+      <c r="A10" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C10" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D10" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E10" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F10" s="6" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="s">
+    <row r="11">
+      <c r="A11" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B11" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C11" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D11" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E11" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F11" s="7" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="7" t="s">
+    <row r="12">
+      <c r="A12" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B12" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D12" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E12" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="F12" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="F6" s="7" t="s">
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="s">
+      <c r="B13" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="D13" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="E13" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="F13" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="E7" s="7" t="s">
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="B14" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="s">
+      <c r="D14" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="C8" s="7" t="s">
+      <c r="E14" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="F14" s="7" t="s">
         <v>233</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>239</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>240</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>246</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="s">
-        <v>248</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>249</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>250</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>251</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="s">
-        <v>254</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>249</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>255</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="s">
-        <v>259</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>249</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>261</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>262</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="s">
-        <v>264</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>249</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>265</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>266</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>267</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -2449,7 +2192,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2464,207 +2207,207 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="C8" s="6" t="s">
         <v>270</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="D8" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="E8" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="E1" s="9" t="s">
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="s">
+      <c r="B9" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C9" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D9" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E9" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="E2" s="7" t="s">
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="C10" s="6" t="s">
         <v>280</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="D10" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="E10" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="E3" s="7" t="s">
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="s">
+      <c r="B11" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C11" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D11" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E11" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="E4" s="7" t="s">
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="s">
+      <c r="B12" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>285</v>
-      </c>
-      <c r="C5" s="7" t="s">
+      <c r="C12" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D12" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="E12" s="6" t="s">
         <v>291</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>293</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>294</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>295</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>296</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="s">
-        <v>298</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>299</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>300</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>301</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="s">
-        <v>303</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>304</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>305</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>306</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="s">
-        <v>308</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>310</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="s">
-        <v>313</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>314</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="s">
-        <v>318</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>319</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>320</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>321</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>324</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>325</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>326</v>
       </c>
     </row>
   </sheetData>
@@ -2672,7 +2415,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2685,115 +2428,115 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>327</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>328</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>329</v>
+      <c r="A1" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>292</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>330</v>
+        <v>295</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>331</v>
+        <v>296</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>332</v>
+        <v>297</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>333</v>
+        <v>298</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>330</v>
+        <v>295</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>334</v>
+        <v>299</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>335</v>
+        <v>300</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>336</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>337</v>
+        <v>302</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>338</v>
+        <v>303</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>339</v>
+        <v>304</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>340</v>
+        <v>305</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>341</v>
+        <v>306</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>342</v>
+        <v>307</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>343</v>
+        <v>308</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>344</v>
+        <v>309</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
-        <v>345</v>
+        <v>310</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>346</v>
+        <v>311</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>347</v>
+        <v>312</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>348</v>
+        <v>313</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
-        <v>349</v>
+        <v>314</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>350</v>
+        <v>315</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>351</v>
+        <v>316</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>352</v>
+        <v>317</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
-        <v>353</v>
+        <v>318</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>354</v>
+        <v>319</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>355</v>
+        <v>320</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>356</v>
+        <v>321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>